<commit_message>
Added uniformD, varReqCostHMS and varReqCost presets
</commit_message>
<xml_diff>
--- a/idea/preset_suites_descriptions.xlsx
+++ b/idea/preset_suites_descriptions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Uni\practice\load-balancing-algorithms\idea\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3754C2F3-997F-4E48-8CCC-293D64F65475}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E11D8E3-B462-4E13-A0D6-426673A4D3EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{1B073830-342D-45B6-9306-A000FEF79D6B}"/>
   </bookViews>
@@ -233,10 +233,10 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -578,10 +578,10 @@
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>15</v>
       </c>
       <c r="F2" t="s">
@@ -598,16 +598,16 @@
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="5"/>
+      <c r="E3" s="6"/>
     </row>
     <row r="4" spans="1:8" ht="39.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>20</v>
       </c>
       <c r="F4" t="s">
@@ -624,16 +624,16 @@
       <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="5"/>
+      <c r="E5" s="6"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F6" t="s">
@@ -650,16 +650,16 @@
       <c r="A7" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="5"/>
+      <c r="E7" s="6"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A8" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="6" t="s">
         <v>22</v>
       </c>
       <c r="F8" t="s">
@@ -673,13 +673,13 @@
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="E9" s="5"/>
+      <c r="E9" s="6"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="D10" t="s">
+      <c r="D10" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="6" t="s">
         <v>23</v>
       </c>
       <c r="F10" t="s">
@@ -693,13 +693,13 @@
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="E11" s="5"/>
+      <c r="E11" s="6"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.5">
       <c r="D12" t="s">
         <v>30</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="6" t="s">
         <v>31</v>
       </c>
     </row>
@@ -708,7 +708,7 @@
         <v>7</v>
       </c>
       <c r="B13" s="2"/>
-      <c r="E13" s="5"/>
+      <c r="E13" s="6"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A14" s="1" t="s">
@@ -720,7 +720,7 @@
       <c r="D14" t="s">
         <v>32</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="E14" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -728,104 +728,98 @@
       <c r="A15" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E15" s="5"/>
+      <c r="E15" s="6"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.5">
       <c r="D16" t="s">
         <v>34</v>
       </c>
-      <c r="E16" s="5" t="s">
+      <c r="E16" s="6" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="17" spans="4:5" x14ac:dyDescent="0.5">
-      <c r="E17" s="5"/>
+      <c r="E17" s="6"/>
     </row>
     <row r="18" spans="4:5" x14ac:dyDescent="0.5">
       <c r="D18" t="s">
         <v>37</v>
       </c>
-      <c r="E18" s="5" t="s">
+      <c r="E18" s="6" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="19" spans="4:5" x14ac:dyDescent="0.5">
-      <c r="E19" s="5"/>
+      <c r="E19" s="6"/>
     </row>
     <row r="20" spans="4:5" x14ac:dyDescent="0.5">
       <c r="D20" t="s">
         <v>38</v>
       </c>
-      <c r="E20" s="5" t="s">
+      <c r="E20" s="6" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="21" spans="4:5" x14ac:dyDescent="0.5">
-      <c r="E21" s="5"/>
+      <c r="E21" s="6"/>
     </row>
     <row r="22" spans="4:5" x14ac:dyDescent="0.5">
       <c r="D22" t="s">
         <v>39</v>
       </c>
-      <c r="E22" s="5" t="s">
+      <c r="E22" s="6" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="23" spans="4:5" x14ac:dyDescent="0.5">
-      <c r="E23" s="5"/>
+      <c r="E23" s="6"/>
     </row>
     <row r="24" spans="4:5" x14ac:dyDescent="0.5">
       <c r="D24" t="s">
         <v>40</v>
       </c>
-      <c r="E24" s="5" t="s">
+      <c r="E24" s="6" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="25" spans="4:5" x14ac:dyDescent="0.5">
-      <c r="E25" s="5"/>
+      <c r="E25" s="6"/>
     </row>
     <row r="26" spans="4:5" x14ac:dyDescent="0.5">
       <c r="D26" t="s">
         <v>41</v>
       </c>
-      <c r="E26" s="5" t="s">
+      <c r="E26" s="6" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="27" spans="4:5" x14ac:dyDescent="0.5">
-      <c r="E27" s="5"/>
+      <c r="E27" s="6"/>
     </row>
     <row r="28" spans="4:5" x14ac:dyDescent="0.5">
       <c r="D28" t="s">
         <v>43</v>
       </c>
-      <c r="E28" s="5" t="s">
+      <c r="E28" s="6" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="29" spans="4:5" x14ac:dyDescent="0.5">
-      <c r="E29" s="5"/>
+      <c r="E29" s="6"/>
     </row>
     <row r="30" spans="4:5" x14ac:dyDescent="0.5">
       <c r="D30" t="s">
         <v>44</v>
       </c>
-      <c r="E30" s="5" t="s">
+      <c r="E30" s="6" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="31" spans="4:5" x14ac:dyDescent="0.5">
-      <c r="E31" s="5"/>
+      <c r="E31" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="E6:E7"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="E8:E9"/>
-    <mergeCell ref="E10:E11"/>
     <mergeCell ref="E26:E27"/>
     <mergeCell ref="E28:E29"/>
     <mergeCell ref="E30:E31"/>
@@ -835,6 +829,12 @@
     <mergeCell ref="E20:E21"/>
     <mergeCell ref="E22:E23"/>
     <mergeCell ref="E24:E25"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="E10:E11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
Added burstNorm and burstNormHMS presets
</commit_message>
<xml_diff>
--- a/idea/preset_suites_descriptions.xlsx
+++ b/idea/preset_suites_descriptions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Uni\practice\load-balancing-algorithms\idea\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E11D8E3-B462-4E13-A0D6-426673A4D3EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF8D478A-42D3-4E60-80C7-8ECE878AA423}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{1B073830-342D-45B6-9306-A000FEF79D6B}"/>
   </bookViews>
@@ -696,7 +696,7 @@
       <c r="E11" s="6"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="D12" t="s">
+      <c r="D12" s="5" t="s">
         <v>30</v>
       </c>
       <c r="E12" s="6" t="s">
@@ -717,7 +717,7 @@
       <c r="B14" t="s">
         <v>10</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="5" t="s">
         <v>32</v>
       </c>
       <c r="E14" s="6" t="s">
@@ -820,6 +820,12 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="E10:E11"/>
     <mergeCell ref="E26:E27"/>
     <mergeCell ref="E28:E29"/>
     <mergeCell ref="E30:E31"/>
@@ -829,12 +835,6 @@
     <mergeCell ref="E20:E21"/>
     <mergeCell ref="E22:E23"/>
     <mergeCell ref="E24:E25"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="E6:E7"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="E8:E9"/>
-    <mergeCell ref="E10:E11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>